<commit_message>
Update to match submitted version
</commit_message>
<xml_diff>
--- a/output/tables/covariateCoefsFormatted.xlsx
+++ b/output/tables/covariateCoefsFormatted.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nis100/tbPatientCosts/tb-lmic-patientcosts-review/output/tables/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hu-my.sharepoint.com/personal/nswartwood_hsph_harvard_edu/Documents/Desktop/nis100/tbPatientCosts/tb-lmic-patientcosts-review/output/tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDF635C7-2B95-B14A-9037-8089258CF0C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{EDF635C7-2B95-B14A-9037-8089258CF0C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE91FC0E-F8AF-854C-9620-6566DDB68946}"/>
   <bookViews>
-    <workbookView xWindow="18740" yWindow="2280" windowWidth="35520" windowHeight="18140" activeTab="2" xr2:uid="{0EA54F60-3D4F-6B46-BC31-C5D89344FEF4}"/>
+    <workbookView xWindow="13580" yWindow="780" windowWidth="36000" windowHeight="22600" xr2:uid="{0EA54F60-3D4F-6B46-BC31-C5D89344FEF4}"/>
   </bookViews>
   <sheets>
     <sheet name="covariateCoefsNew" sheetId="1" r:id="rId1"/>
@@ -859,6 +859,9 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -871,9 +874,6 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1271,17 +1271,17 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>1.02</v>
+        <v>0.99</v>
       </c>
       <c r="C2">
-        <v>0.55000000000000004</v>
+        <v>0.53</v>
       </c>
       <c r="D2">
-        <v>1.99</v>
+        <v>1.92</v>
       </c>
       <c r="F2" t="str">
         <f>_xlfn.CONCAT(B2, " ( ", C2, ", ", D2, ")")</f>
-        <v>1.02 ( 0.55, 1.99)</v>
+        <v>0.99 ( 0.53, 1.92)</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -1292,14 +1292,14 @@
         <v>1.84</v>
       </c>
       <c r="C3">
-        <v>0.92</v>
+        <v>0.96</v>
       </c>
       <c r="D3">
-        <v>3.79</v>
+        <v>3.66</v>
       </c>
       <c r="F3" t="str">
         <f t="shared" ref="F3:F46" si="0">_xlfn.CONCAT(B3, " ( ", C3, ", ", D3, ")")</f>
-        <v>1.84 ( 0.92, 3.79)</v>
+        <v>1.84 ( 0.96, 3.66)</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -1307,17 +1307,17 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>1.27</v>
+        <v>1.36</v>
       </c>
       <c r="C4">
-        <v>0.49</v>
+        <v>0.53</v>
       </c>
       <c r="D4">
-        <v>3.47</v>
+        <v>3.57</v>
       </c>
       <c r="F4" t="str">
         <f t="shared" si="0"/>
-        <v>1.27 ( 0.49, 3.47)</v>
+        <v>1.36 ( 0.53, 3.57)</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -1325,17 +1325,17 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>2.76</v>
+        <v>2.5</v>
       </c>
       <c r="C5">
-        <v>0.89</v>
+        <v>0.77</v>
       </c>
       <c r="D5">
-        <v>8.1300000000000008</v>
+        <v>7.47</v>
       </c>
       <c r="F5" t="str">
         <f t="shared" si="0"/>
-        <v>2.76 ( 0.89, 8.13)</v>
+        <v>2.5 ( 0.77, 7.47)</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -1343,17 +1343,17 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>9.23</v>
+        <v>7.6</v>
       </c>
       <c r="C6">
-        <v>1.1599999999999999</v>
+        <v>1.22</v>
       </c>
       <c r="D6">
-        <v>87.58</v>
+        <v>58.49</v>
       </c>
       <c r="F6" t="str">
         <f t="shared" si="0"/>
-        <v>9.23 ( 1.16, 87.58)</v>
+        <v>7.6 ( 1.22, 58.49)</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -1361,17 +1361,17 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>7.26</v>
+        <v>7.39</v>
       </c>
       <c r="C7">
-        <v>2.83</v>
+        <v>2.92</v>
       </c>
       <c r="D7">
-        <v>17.68</v>
+        <v>19.440000000000001</v>
       </c>
       <c r="F7" t="str">
         <f t="shared" si="0"/>
-        <v>7.26 ( 2.83, 17.68)</v>
+        <v>7.39 ( 2.92, 19.44)</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -1379,17 +1379,17 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>4.6900000000000004</v>
+        <v>4.05</v>
       </c>
       <c r="C8">
-        <v>1.67</v>
+        <v>1.39</v>
       </c>
       <c r="D8">
-        <v>22.09</v>
+        <v>17.59</v>
       </c>
       <c r="F8" t="str">
         <f t="shared" si="0"/>
-        <v>4.69 ( 1.67, 22.09)</v>
+        <v>4.05 ( 1.39, 17.59)</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -1397,17 +1397,17 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>7.89</v>
+        <v>6.89</v>
       </c>
       <c r="C9">
-        <v>3.1</v>
+        <v>2.91</v>
       </c>
       <c r="D9">
-        <v>16.559999999999999</v>
+        <v>17.18</v>
       </c>
       <c r="F9" t="str">
         <f t="shared" si="0"/>
-        <v>7.89 ( 3.1, 16.56)</v>
+        <v>6.89 ( 2.91, 17.18)</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -1415,17 +1415,17 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>7.25</v>
+        <v>5.92</v>
       </c>
       <c r="C10">
-        <v>3.05</v>
+        <v>2.5099999999999998</v>
       </c>
       <c r="D10">
-        <v>16.36</v>
+        <v>13.67</v>
       </c>
       <c r="F10" t="str">
         <f t="shared" si="0"/>
-        <v>7.25 ( 3.05, 16.36)</v>
+        <v>5.92 ( 2.51, 13.67)</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -1433,17 +1433,17 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>1.18</v>
+        <v>1.36</v>
       </c>
       <c r="C11">
-        <v>0.85</v>
+        <v>1</v>
       </c>
       <c r="D11">
-        <v>1.63</v>
+        <v>1.89</v>
       </c>
       <c r="F11" t="str">
         <f t="shared" si="0"/>
-        <v>1.18 ( 0.85, 1.63)</v>
+        <v>1.36 ( 1, 1.89)</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -1451,17 +1451,17 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>1.07</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="C12">
         <v>0.81</v>
       </c>
       <c r="D12">
-        <v>1.39</v>
+        <v>1.48</v>
       </c>
       <c r="F12" t="str">
         <f t="shared" si="0"/>
-        <v>1.07 ( 0.81, 1.39)</v>
+        <v>1.1 ( 0.81, 1.48)</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -1469,17 +1469,17 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>1.38</v>
+        <v>1.59</v>
       </c>
       <c r="C13">
-        <v>0.92</v>
+        <v>1.03</v>
       </c>
       <c r="D13">
-        <v>2.4</v>
+        <v>2.7</v>
       </c>
       <c r="F13" t="str">
         <f t="shared" si="0"/>
-        <v>1.38 ( 0.92, 2.4)</v>
+        <v>1.59 ( 1.03, 2.7)</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -1487,17 +1487,17 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>0.96</v>
+        <v>1.06</v>
       </c>
       <c r="C14">
-        <v>0.55000000000000004</v>
+        <v>0.61</v>
       </c>
       <c r="D14">
-        <v>1.45</v>
+        <v>1.71</v>
       </c>
       <c r="F14" t="str">
         <f t="shared" si="0"/>
-        <v>0.96 ( 0.55, 1.45)</v>
+        <v>1.06 ( 0.61, 1.71)</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
@@ -1505,17 +1505,17 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="C15">
         <v>0.4</v>
       </c>
       <c r="D15">
-        <v>2.02</v>
+        <v>1.97</v>
       </c>
       <c r="F15" t="str">
         <f t="shared" si="0"/>
-        <v>1 ( 0.4, 2.02)</v>
+        <v>1.02 ( 0.4, 1.97)</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
@@ -1523,17 +1523,17 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="C16">
-        <v>0.5</v>
+        <v>0.51</v>
       </c>
       <c r="D16">
-        <v>1.43</v>
+        <v>1.55</v>
       </c>
       <c r="F16" t="str">
         <f t="shared" si="0"/>
-        <v>0.98 ( 0.5, 1.43)</v>
+        <v>0.99 ( 0.51, 1.55)</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -1541,17 +1541,17 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>1.01</v>
+        <v>1.1399999999999999</v>
       </c>
       <c r="C17">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="D17">
-        <v>1.58</v>
+        <v>1.85</v>
       </c>
       <c r="F17" t="str">
         <f t="shared" si="0"/>
-        <v>1.01 ( 0.6, 1.58)</v>
+        <v>1.14 ( 0.7, 1.85)</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -1559,17 +1559,17 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>1.04</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="C18">
-        <v>0.64</v>
+        <v>0.76</v>
       </c>
       <c r="D18">
-        <v>1.46</v>
+        <v>1.7</v>
       </c>
       <c r="F18" t="str">
         <f t="shared" si="0"/>
-        <v>1.04 ( 0.64, 1.46)</v>
+        <v>1.15 ( 0.76, 1.7)</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
@@ -1577,17 +1577,17 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>1.08</v>
+        <v>1.22</v>
       </c>
       <c r="C19">
-        <v>0.67</v>
+        <v>0.8</v>
       </c>
       <c r="D19">
-        <v>1.66</v>
+        <v>1.84</v>
       </c>
       <c r="F19" t="str">
         <f t="shared" si="0"/>
-        <v>1.08 ( 0.67, 1.66)</v>
+        <v>1.22 ( 0.8, 1.84)</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
@@ -1595,17 +1595,17 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>2.1800000000000002</v>
+        <v>1.36</v>
       </c>
       <c r="C20">
-        <v>1.2</v>
+        <v>0.86</v>
       </c>
       <c r="D20">
-        <v>3.89</v>
+        <v>2.19</v>
       </c>
       <c r="F20" t="str">
         <f t="shared" si="0"/>
-        <v>2.18 ( 1.2, 3.89)</v>
+        <v>1.36 ( 0.86, 2.19)</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
@@ -1613,17 +1613,17 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>1.59</v>
+        <v>1.1299999999999999</v>
       </c>
       <c r="C21">
-        <v>0.87</v>
+        <v>0.73</v>
       </c>
       <c r="D21">
-        <v>2.78</v>
+        <v>1.73</v>
       </c>
       <c r="F21" t="str">
         <f t="shared" si="0"/>
-        <v>1.59 ( 0.87, 2.78)</v>
+        <v>1.13 ( 0.73, 1.73)</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
@@ -1631,17 +1631,17 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>1.56</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="C22">
-        <v>0.84</v>
+        <v>0.68</v>
       </c>
       <c r="D22">
-        <v>3.02</v>
+        <v>1.74</v>
       </c>
       <c r="F22" t="str">
         <f t="shared" si="0"/>
-        <v>1.56 ( 0.84, 3.02)</v>
+        <v>1.1 ( 0.68, 1.74)</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
@@ -1649,17 +1649,17 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>1.91</v>
+        <v>1.18</v>
       </c>
       <c r="C23">
-        <v>0.97</v>
+        <v>0.69</v>
       </c>
       <c r="D23">
-        <v>4.75</v>
+        <v>2.1</v>
       </c>
       <c r="F23" t="str">
         <f t="shared" si="0"/>
-        <v>1.91 ( 0.97, 4.75)</v>
+        <v>1.18 ( 0.69, 2.1)</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
@@ -1667,17 +1667,17 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>1.69</v>
+        <v>1.08</v>
       </c>
       <c r="C24">
-        <v>0.62</v>
+        <v>0.54</v>
       </c>
       <c r="D24">
-        <v>5.3</v>
+        <v>2.06</v>
       </c>
       <c r="F24" t="str">
         <f t="shared" si="0"/>
-        <v>1.69 ( 0.62, 5.3)</v>
+        <v>1.08 ( 0.54, 2.06)</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
@@ -1685,17 +1685,17 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>2.16</v>
+        <v>1.34</v>
       </c>
       <c r="C25">
-        <v>0.98</v>
+        <v>0.76</v>
       </c>
       <c r="D25">
-        <v>4.96</v>
+        <v>2.72</v>
       </c>
       <c r="F25" t="str">
         <f t="shared" si="0"/>
-        <v>2.16 ( 0.98, 4.96)</v>
+        <v>1.34 ( 0.76, 2.72)</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
@@ -1703,17 +1703,17 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>3.35</v>
+        <v>1.4</v>
       </c>
       <c r="C26">
-        <v>1.27</v>
+        <v>0.76</v>
       </c>
       <c r="D26">
-        <v>23.65</v>
+        <v>3.85</v>
       </c>
       <c r="F26" t="str">
         <f t="shared" si="0"/>
-        <v>3.35 ( 1.27, 23.65)</v>
+        <v>1.4 ( 0.76, 3.85)</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
@@ -1721,17 +1721,17 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>1.25</v>
+        <v>0.96</v>
       </c>
       <c r="C27">
-        <v>0.63</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="D27">
-        <v>2.5499999999999998</v>
+        <v>1.54</v>
       </c>
       <c r="F27" t="str">
         <f t="shared" si="0"/>
-        <v>1.25 ( 0.63, 2.55)</v>
+        <v>0.96 ( 0.58, 1.54)</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
@@ -1739,17 +1739,17 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>1.63</v>
+        <v>1.1399999999999999</v>
       </c>
       <c r="C28">
-        <v>0.81</v>
+        <v>0.68</v>
       </c>
       <c r="D28">
-        <v>3.28</v>
+        <v>1.86</v>
       </c>
       <c r="F28" t="str">
         <f t="shared" si="0"/>
-        <v>1.63 ( 0.81, 3.28)</v>
+        <v>1.14 ( 0.68, 1.86)</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
@@ -1757,17 +1757,17 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>1.66</v>
+        <v>1.77</v>
       </c>
       <c r="C29">
-        <v>1.1299999999999999</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="D29">
-        <v>2.39</v>
+        <v>2.72</v>
       </c>
       <c r="F29" t="str">
         <f t="shared" si="0"/>
-        <v>1.66 ( 1.13, 2.39)</v>
+        <v>1.77 ( 1.15, 2.72)</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
@@ -1775,17 +1775,17 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>1.41</v>
+        <v>1.39</v>
       </c>
       <c r="C30">
-        <v>1.01</v>
+        <v>0.99</v>
       </c>
       <c r="D30">
-        <v>1.9</v>
+        <v>1.98</v>
       </c>
       <c r="F30" t="str">
         <f t="shared" si="0"/>
-        <v>1.41 ( 1.01, 1.9)</v>
+        <v>1.39 ( 0.99, 1.98)</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
@@ -1793,17 +1793,17 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>1.18</v>
+        <v>1.34</v>
       </c>
       <c r="C31">
-        <v>0.8</v>
+        <v>0.85</v>
       </c>
       <c r="D31">
-        <v>1.77</v>
+        <v>2.09</v>
       </c>
       <c r="F31" t="str">
         <f t="shared" si="0"/>
-        <v>1.18 ( 0.8, 1.77)</v>
+        <v>1.34 ( 0.85, 2.09)</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
@@ -1814,14 +1814,14 @@
         <v>1.31</v>
       </c>
       <c r="C32">
-        <v>0.77</v>
+        <v>0.7</v>
       </c>
       <c r="D32">
-        <v>2.46</v>
+        <v>2.68</v>
       </c>
       <c r="F32" t="str">
         <f t="shared" si="0"/>
-        <v>1.31 ( 0.77, 2.46)</v>
+        <v>1.31 ( 0.7, 2.68)</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
@@ -1829,17 +1829,17 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>0.89</v>
+        <v>0.85</v>
       </c>
       <c r="C33">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="D33">
         <v>2.08</v>
       </c>
       <c r="F33" t="str">
         <f t="shared" si="0"/>
-        <v>0.89 ( 0.26, 2.08)</v>
+        <v>0.85 ( 0.25, 2.08)</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
@@ -1847,17 +1847,17 @@
         <v>33</v>
       </c>
       <c r="B34">
-        <v>0.76</v>
+        <v>0.77</v>
       </c>
       <c r="C34">
         <v>0.45</v>
       </c>
       <c r="D34">
-        <v>1.2</v>
+        <v>1.33</v>
       </c>
       <c r="F34" t="str">
         <f t="shared" si="0"/>
-        <v>0.76 ( 0.45, 1.2)</v>
+        <v>0.77 ( 0.45, 1.33)</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
@@ -1865,17 +1865,17 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>1.26</v>
+        <v>1.03</v>
       </c>
       <c r="C35">
-        <v>0.65</v>
+        <v>0.51</v>
       </c>
       <c r="D35">
-        <v>2.67</v>
+        <v>2.08</v>
       </c>
       <c r="F35" t="str">
         <f t="shared" si="0"/>
-        <v>1.26 ( 0.65, 2.67)</v>
+        <v>1.03 ( 0.51, 2.08)</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
@@ -1883,17 +1883,17 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>0.61</v>
+        <v>0.62</v>
       </c>
       <c r="C36">
-        <v>0.37</v>
+        <v>0.38</v>
       </c>
       <c r="D36">
-        <v>1.1100000000000001</v>
+        <v>1.18</v>
       </c>
       <c r="F36" t="str">
         <f t="shared" si="0"/>
-        <v>0.61 ( 0.37, 1.11)</v>
+        <v>0.62 ( 0.38, 1.18)</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
@@ -1904,14 +1904,14 @@
         <v>0.75</v>
       </c>
       <c r="C37">
-        <v>0.49</v>
+        <v>0.47</v>
       </c>
       <c r="D37">
-        <v>1.18</v>
+        <v>1.21</v>
       </c>
       <c r="F37" t="str">
         <f t="shared" si="0"/>
-        <v>0.75 ( 0.49, 1.18)</v>
+        <v>0.75 ( 0.47, 1.21)</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
@@ -1919,17 +1919,17 @@
         <v>37</v>
       </c>
       <c r="B38">
-        <v>0.85</v>
+        <v>1.0900000000000001</v>
       </c>
       <c r="C38">
-        <v>0.48</v>
+        <v>0.7</v>
       </c>
       <c r="D38">
-        <v>1.58</v>
+        <v>1.7</v>
       </c>
       <c r="F38" t="str">
         <f t="shared" si="0"/>
-        <v>0.85 ( 0.48, 1.58)</v>
+        <v>1.09 ( 0.7, 1.7)</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
@@ -1937,17 +1937,17 @@
         <v>38</v>
       </c>
       <c r="B39">
-        <v>0.81</v>
+        <v>1.1399999999999999</v>
       </c>
       <c r="C39">
-        <v>0.46</v>
+        <v>0.75</v>
       </c>
       <c r="D39">
-        <v>1.43</v>
+        <v>1.73</v>
       </c>
       <c r="F39" t="str">
         <f t="shared" si="0"/>
-        <v>0.81 ( 0.46, 1.43)</v>
+        <v>1.14 ( 0.75, 1.73)</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
@@ -1955,17 +1955,17 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>0.81</v>
+        <v>1.19</v>
       </c>
       <c r="C40">
-        <v>0.44</v>
+        <v>0.76</v>
       </c>
       <c r="D40">
-        <v>1.44</v>
+        <v>1.91</v>
       </c>
       <c r="F40" t="str">
         <f t="shared" si="0"/>
-        <v>0.81 ( 0.44, 1.44)</v>
+        <v>1.19 ( 0.76, 1.91)</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
@@ -1973,17 +1973,17 @@
         <v>40</v>
       </c>
       <c r="B41">
-        <v>0.78</v>
+        <v>1.17</v>
       </c>
       <c r="C41">
-        <v>0.37</v>
+        <v>0.68</v>
       </c>
       <c r="D41">
-        <v>1.38</v>
+        <v>2.1800000000000002</v>
       </c>
       <c r="F41" t="str">
         <f t="shared" si="0"/>
-        <v>0.78 ( 0.37, 1.38)</v>
+        <v>1.17 ( 0.68, 2.18)</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
@@ -1991,17 +1991,17 @@
         <v>41</v>
       </c>
       <c r="B42">
-        <v>0.82</v>
+        <v>0.81</v>
       </c>
       <c r="C42">
-        <v>0.43</v>
+        <v>0.33</v>
       </c>
       <c r="D42">
-        <v>1.7</v>
+        <v>1.64</v>
       </c>
       <c r="F42" t="str">
         <f t="shared" si="0"/>
-        <v>0.82 ( 0.43, 1.7)</v>
+        <v>0.81 ( 0.33, 1.64)</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
@@ -2009,17 +2009,17 @@
         <v>42</v>
       </c>
       <c r="B43">
-        <v>0.86</v>
+        <v>1.02</v>
       </c>
       <c r="C43">
-        <v>0.45</v>
+        <v>0.63</v>
       </c>
       <c r="D43">
-        <v>1.63</v>
+        <v>1.65</v>
       </c>
       <c r="F43" t="str">
         <f t="shared" si="0"/>
-        <v>0.86 ( 0.45, 1.63)</v>
+        <v>1.02 ( 0.63, 1.65)</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
@@ -2027,17 +2027,17 @@
         <v>43</v>
       </c>
       <c r="B44">
-        <v>0.86</v>
+        <v>1.62</v>
       </c>
       <c r="C44">
-        <v>0.47</v>
+        <v>0.88</v>
       </c>
       <c r="D44">
-        <v>2.11</v>
+        <v>3.78</v>
       </c>
       <c r="F44" t="str">
         <f t="shared" si="0"/>
-        <v>0.86 ( 0.47, 2.11)</v>
+        <v>1.62 ( 0.88, 3.78)</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
@@ -2045,17 +2045,17 @@
         <v>44</v>
       </c>
       <c r="B45">
-        <v>0.81</v>
+        <v>0.76</v>
       </c>
       <c r="C45">
-        <v>0.42</v>
+        <v>0.46</v>
       </c>
       <c r="D45">
-        <v>1.47</v>
+        <v>1.21</v>
       </c>
       <c r="F45" t="str">
         <f t="shared" si="0"/>
-        <v>0.81 ( 0.42, 1.47)</v>
+        <v>0.76 ( 0.46, 1.21)</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
@@ -2063,17 +2063,17 @@
         <v>45</v>
       </c>
       <c r="B46">
-        <v>0.86</v>
+        <v>0.84</v>
       </c>
       <c r="C46">
-        <v>0.46</v>
+        <v>0.52</v>
       </c>
       <c r="D46">
-        <v>1.57</v>
+        <v>1.32</v>
       </c>
       <c r="F46" t="str">
         <f t="shared" si="0"/>
-        <v>0.86 ( 0.46, 1.57)</v>
+        <v>0.84 ( 0.52, 1.32)</v>
       </c>
     </row>
   </sheetData>
@@ -2094,17 +2094,17 @@
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="2"/>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
     </row>
     <row r="3" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="3"/>
@@ -2124,15 +2124,15 @@
       </c>
       <c r="B5" s="11" t="str">
         <f>covariateCoefsNew!F2</f>
-        <v>1.02 ( 0.55, 1.99)</v>
+        <v>0.99 ( 0.53, 1.92)</v>
       </c>
       <c r="C5" s="12" t="str">
         <f>covariateCoefsNew!F3</f>
-        <v>1.84 ( 0.92, 3.79)</v>
+        <v>1.84 ( 0.96, 3.66)</v>
       </c>
       <c r="D5" s="7" t="str">
         <f>covariateCoefsNew!F4</f>
-        <v>1.27 ( 0.49, 3.47)</v>
+        <v>1.36 ( 0.53, 3.57)</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -2141,15 +2141,15 @@
       </c>
       <c r="B6" s="11" t="str">
         <f>covariateCoefsNew!F11</f>
-        <v>1.18 ( 0.85, 1.63)</v>
+        <v>1.36 ( 1, 1.89)</v>
       </c>
       <c r="C6" s="12" t="str">
         <f>covariateCoefsNew!F12</f>
-        <v>1.07 ( 0.81, 1.39)</v>
+        <v>1.1 ( 0.81, 1.48)</v>
       </c>
       <c r="D6" s="7" t="str">
         <f>covariateCoefsNew!F13</f>
-        <v>1.38 ( 0.92, 2.4)</v>
+        <v>1.59 ( 1.03, 2.7)</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -2158,15 +2158,15 @@
       </c>
       <c r="B7" s="11" t="str">
         <f>covariateCoefsNew!F20</f>
-        <v>2.18 ( 1.2, 3.89)</v>
+        <v>1.36 ( 0.86, 2.19)</v>
       </c>
       <c r="C7" s="12" t="str">
         <f>covariateCoefsNew!F21</f>
-        <v>1.59 ( 0.87, 2.78)</v>
+        <v>1.13 ( 0.73, 1.73)</v>
       </c>
       <c r="D7" s="7" t="str">
         <f>covariateCoefsNew!F22</f>
-        <v>1.56 ( 0.84, 3.02)</v>
+        <v>1.1 ( 0.68, 1.74)</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -2175,15 +2175,15 @@
       </c>
       <c r="B8" s="11" t="str">
         <f>covariateCoefsNew!F29</f>
-        <v>1.66 ( 1.13, 2.39)</v>
+        <v>1.77 ( 1.15, 2.72)</v>
       </c>
       <c r="C8" s="12" t="str">
         <f>covariateCoefsNew!F30</f>
-        <v>1.41 ( 1.01, 1.9)</v>
+        <v>1.39 ( 0.99, 1.98)</v>
       </c>
       <c r="D8" s="7" t="str">
         <f>covariateCoefsNew!F31</f>
-        <v>1.18 ( 0.8, 1.77)</v>
+        <v>1.34 ( 0.85, 2.09)</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -2192,15 +2192,15 @@
       </c>
       <c r="B9" s="11" t="str">
         <f>covariateCoefsNew!F38</f>
-        <v>0.85 ( 0.48, 1.58)</v>
+        <v>1.09 ( 0.7, 1.7)</v>
       </c>
       <c r="C9" s="12" t="str">
         <f>covariateCoefsNew!F39</f>
-        <v>0.81 ( 0.46, 1.43)</v>
+        <v>1.14 ( 0.75, 1.73)</v>
       </c>
       <c r="D9" s="7" t="str">
         <f>covariateCoefsNew!F40</f>
-        <v>0.81 ( 0.44, 1.44)</v>
+        <v>1.19 ( 0.76, 1.91)</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -2211,11 +2211,11 @@
     </row>
     <row r="11" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="17"/>
-      <c r="D11" s="19"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="22"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="3"/>
@@ -2235,15 +2235,15 @@
       </c>
       <c r="B13" s="11" t="str">
         <f>covariateCoefsNew!F5</f>
-        <v>2.76 ( 0.89, 8.13)</v>
+        <v>2.5 ( 0.77, 7.47)</v>
       </c>
       <c r="C13" s="12" t="str">
         <f>covariateCoefsNew!F6</f>
-        <v>9.23 ( 1.16, 87.58)</v>
+        <v>7.6 ( 1.22, 58.49)</v>
       </c>
       <c r="D13" s="7" t="str">
         <f>covariateCoefsNew!F7</f>
-        <v>7.26 ( 2.83, 17.68)</v>
+        <v>7.39 ( 2.92, 19.44)</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
@@ -2252,15 +2252,15 @@
       </c>
       <c r="B14" s="11" t="str">
         <f>covariateCoefsNew!F14</f>
-        <v>0.96 ( 0.55, 1.45)</v>
+        <v>1.06 ( 0.61, 1.71)</v>
       </c>
       <c r="C14" s="12" t="str">
         <f>covariateCoefsNew!F15</f>
-        <v>1 ( 0.4, 2.02)</v>
+        <v>1.02 ( 0.4, 1.97)</v>
       </c>
       <c r="D14" s="7" t="str">
         <f>covariateCoefsNew!F16</f>
-        <v>0.98 ( 0.5, 1.43)</v>
+        <v>0.99 ( 0.51, 1.55)</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
@@ -2269,15 +2269,15 @@
       </c>
       <c r="B15" s="11" t="str">
         <f>covariateCoefsNew!F23</f>
-        <v>1.91 ( 0.97, 4.75)</v>
+        <v>1.18 ( 0.69, 2.1)</v>
       </c>
       <c r="C15" s="12" t="str">
         <f>covariateCoefsNew!F24</f>
-        <v>1.69 ( 0.62, 5.3)</v>
+        <v>1.08 ( 0.54, 2.06)</v>
       </c>
       <c r="D15" s="7" t="str">
         <f>covariateCoefsNew!F25</f>
-        <v>2.16 ( 0.98, 4.96)</v>
+        <v>1.34 ( 0.76, 2.72)</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
@@ -2286,15 +2286,15 @@
       </c>
       <c r="B16" s="11" t="str">
         <f>covariateCoefsNew!F32</f>
-        <v>1.31 ( 0.77, 2.46)</v>
+        <v>1.31 ( 0.7, 2.68)</v>
       </c>
       <c r="C16" s="12" t="str">
         <f>covariateCoefsNew!F33</f>
-        <v>0.89 ( 0.26, 2.08)</v>
+        <v>0.85 ( 0.25, 2.08)</v>
       </c>
       <c r="D16" s="7" t="str">
         <f>covariateCoefsNew!F34</f>
-        <v>0.76 ( 0.45, 1.2)</v>
+        <v>0.77 ( 0.45, 1.33)</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
@@ -2303,15 +2303,15 @@
       </c>
       <c r="B17" s="11" t="str">
         <f>covariateCoefsNew!F41</f>
-        <v>0.78 ( 0.37, 1.38)</v>
+        <v>1.17 ( 0.68, 2.18)</v>
       </c>
       <c r="C17" s="12" t="str">
         <f>covariateCoefsNew!F42</f>
-        <v>0.82 ( 0.43, 1.7)</v>
+        <v>0.81 ( 0.33, 1.64)</v>
       </c>
       <c r="D17" s="7" t="str">
         <f>covariateCoefsNew!F43</f>
-        <v>0.86 ( 0.45, 1.63)</v>
+        <v>1.02 ( 0.63, 1.65)</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -2322,11 +2322,11 @@
     </row>
     <row r="19" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
-      <c r="B19" s="18" t="s">
+      <c r="B19" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="C19" s="17"/>
-      <c r="D19" s="19"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="22"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="3"/>
@@ -2346,15 +2346,15 @@
       </c>
       <c r="B21" s="11" t="str">
         <f>covariateCoefsNew!F8</f>
-        <v>4.69 ( 1.67, 22.09)</v>
+        <v>4.05 ( 1.39, 17.59)</v>
       </c>
       <c r="C21" s="12" t="str">
         <f>covariateCoefsNew!F9</f>
-        <v>7.89 ( 3.1, 16.56)</v>
+        <v>6.89 ( 2.91, 17.18)</v>
       </c>
       <c r="D21" s="7" t="str">
         <f>covariateCoefsNew!F10</f>
-        <v>7.25 ( 3.05, 16.36)</v>
+        <v>5.92 ( 2.51, 13.67)</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
@@ -2363,15 +2363,15 @@
       </c>
       <c r="B22" s="11" t="str">
         <f>covariateCoefsNew!F17</f>
-        <v>1.01 ( 0.6, 1.58)</v>
+        <v>1.14 ( 0.7, 1.85)</v>
       </c>
       <c r="C22" s="12" t="str">
         <f>covariateCoefsNew!F18</f>
-        <v>1.04 ( 0.64, 1.46)</v>
+        <v>1.15 ( 0.76, 1.7)</v>
       </c>
       <c r="D22" s="7" t="str">
         <f>covariateCoefsNew!F19</f>
-        <v>1.08 ( 0.67, 1.66)</v>
+        <v>1.22 ( 0.8, 1.84)</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
@@ -2380,15 +2380,15 @@
       </c>
       <c r="B23" s="11" t="str">
         <f>covariateCoefsNew!F26</f>
-        <v>3.35 ( 1.27, 23.65)</v>
+        <v>1.4 ( 0.76, 3.85)</v>
       </c>
       <c r="C23" s="12" t="str">
         <f>covariateCoefsNew!F27</f>
-        <v>1.25 ( 0.63, 2.55)</v>
+        <v>0.96 ( 0.58, 1.54)</v>
       </c>
       <c r="D23" s="7" t="str">
         <f>covariateCoefsNew!F28</f>
-        <v>1.63 ( 0.81, 3.28)</v>
+        <v>1.14 ( 0.68, 1.86)</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
@@ -2397,15 +2397,15 @@
       </c>
       <c r="B24" s="11" t="str">
         <f>covariateCoefsNew!F35</f>
-        <v>1.26 ( 0.65, 2.67)</v>
+        <v>1.03 ( 0.51, 2.08)</v>
       </c>
       <c r="C24" s="12" t="str">
         <f>covariateCoefsNew!F36</f>
-        <v>0.61 ( 0.37, 1.11)</v>
+        <v>0.62 ( 0.38, 1.18)</v>
       </c>
       <c r="D24" s="7" t="str">
         <f>covariateCoefsNew!F37</f>
-        <v>0.75 ( 0.49, 1.18)</v>
+        <v>0.75 ( 0.47, 1.21)</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -2414,15 +2414,15 @@
       </c>
       <c r="B25" s="15" t="str">
         <f>covariateCoefsNew!F44</f>
-        <v>0.86 ( 0.47, 2.11)</v>
+        <v>1.62 ( 0.88, 3.78)</v>
       </c>
       <c r="C25" s="8" t="str">
         <f>covariateCoefsNew!F45</f>
-        <v>0.81 ( 0.42, 1.47)</v>
+        <v>0.76 ( 0.46, 1.21)</v>
       </c>
       <c r="D25" s="9" t="str">
         <f>covariateCoefsNew!F46</f>
-        <v>0.86 ( 0.46, 1.57)</v>
+        <v>0.84 ( 0.52, 1.32)</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
@@ -2451,21 +2451,21 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="16" t="s">
         <v>15</v>
       </c>
       <c r="B3">
         <f>covariateCoefsNew!B2</f>
-        <v>1.02</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="16" t="s">
         <v>16</v>
       </c>
       <c r="B4">
@@ -2474,279 +2474,279 @@
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="17" t="s">
         <v>17</v>
       </c>
       <c r="B5">
         <f>covariateCoefsNew!B4</f>
-        <v>1.27</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="16" t="s">
         <v>18</v>
       </c>
       <c r="B6">
         <f>covariateCoefsNew!B5</f>
-        <v>2.76</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="16" t="s">
         <v>19</v>
       </c>
       <c r="B7">
         <f>covariateCoefsNew!B6</f>
-        <v>9.23</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="17" t="s">
         <v>20</v>
       </c>
       <c r="B8">
         <f>covariateCoefsNew!B7</f>
-        <v>7.26</v>
+        <v>7.39</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" s="20" t="s">
+      <c r="A9" s="16" t="s">
         <v>21</v>
       </c>
       <c r="B9">
         <f>covariateCoefsNew!B8</f>
-        <v>4.6900000000000004</v>
+        <v>4.05</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="16" t="s">
         <v>22</v>
       </c>
       <c r="B10">
         <f>covariateCoefsNew!B9</f>
-        <v>7.89</v>
+        <v>6.89</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="17" t="s">
         <v>23</v>
       </c>
       <c r="B11">
         <f>covariateCoefsNew!B10</f>
-        <v>7.25</v>
+        <v>5.92</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" s="20" t="s">
+      <c r="A12" s="16" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" s="20" t="s">
+      <c r="A13" s="16" t="s">
         <v>25</v>
       </c>
       <c r="B13">
         <f>covariateCoefsNew!B11</f>
-        <v>1.18</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14" s="20" t="s">
+      <c r="A14" s="16" t="s">
         <v>26</v>
       </c>
       <c r="B14">
         <f>covariateCoefsNew!B12</f>
-        <v>1.07</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A15" s="21" t="s">
+      <c r="A15" s="17" t="s">
         <v>27</v>
       </c>
       <c r="B15">
         <f>covariateCoefsNew!B13</f>
-        <v>1.38</v>
+        <v>1.59</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16" s="20" t="s">
+      <c r="A16" s="16" t="s">
         <v>28</v>
       </c>
       <c r="B16">
         <f>covariateCoefsNew!B14</f>
-        <v>0.96</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" s="20" t="s">
+      <c r="A17" s="16" t="s">
         <v>29</v>
       </c>
       <c r="B17">
         <f>covariateCoefsNew!B15</f>
-        <v>1</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="17" t="s">
         <v>30</v>
       </c>
       <c r="B18">
         <f>covariateCoefsNew!B16</f>
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" s="20" t="s">
+      <c r="A19" s="16" t="s">
         <v>31</v>
       </c>
       <c r="B19">
         <f>covariateCoefsNew!B17</f>
-        <v>1.01</v>
+        <v>1.1399999999999999</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20" s="20" t="s">
+      <c r="A20" s="16" t="s">
         <v>32</v>
       </c>
       <c r="B20">
         <f>covariateCoefsNew!B18</f>
-        <v>1.04</v>
+        <v>1.1499999999999999</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="17" t="s">
         <v>33</v>
       </c>
       <c r="B21">
         <f>covariateCoefsNew!B19</f>
-        <v>1.08</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" s="20" t="s">
+      <c r="A22" s="16" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A23" s="20" t="s">
+      <c r="A23" s="16" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A24" s="20" t="s">
+      <c r="A24" s="16" t="s">
         <v>36</v>
       </c>
       <c r="B24">
         <f>covariateCoefsNew!B20</f>
-        <v>2.1800000000000002</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A25" s="20" t="s">
+      <c r="A25" s="16" t="s">
         <v>37</v>
       </c>
       <c r="B25">
         <f>covariateCoefsNew!B21</f>
-        <v>1.59</v>
+        <v>1.1299999999999999</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A26" s="20" t="s">
+      <c r="A26" s="16" t="s">
         <v>38</v>
       </c>
       <c r="B26">
         <f>covariateCoefsNew!B22</f>
-        <v>1.56</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A27" s="20" t="s">
+      <c r="A27" s="16" t="s">
         <v>39</v>
       </c>
       <c r="B27">
         <f>covariateCoefsNew!B23</f>
-        <v>1.91</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A28" s="20" t="s">
+      <c r="A28" s="16" t="s">
         <v>40</v>
       </c>
       <c r="B28">
         <f>covariateCoefsNew!B24</f>
-        <v>1.69</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A29" s="20" t="s">
+      <c r="A29" s="16" t="s">
         <v>41</v>
       </c>
       <c r="B29">
         <f>covariateCoefsNew!B25</f>
-        <v>2.16</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A30" s="20" t="s">
+      <c r="A30" s="16" t="s">
         <v>42</v>
       </c>
       <c r="B30">
         <f>covariateCoefsNew!B26</f>
-        <v>3.35</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A31" s="20" t="s">
+      <c r="A31" s="16" t="s">
         <v>43</v>
       </c>
       <c r="B31">
         <f>covariateCoefsNew!B27</f>
-        <v>1.25</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A32" s="20" t="s">
+      <c r="A32" s="16" t="s">
         <v>44</v>
       </c>
       <c r="B32">
         <f>covariateCoefsNew!B28</f>
-        <v>1.63</v>
+        <v>1.1399999999999999</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A33" s="20" t="s">
+      <c r="A33" s="16" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A34" s="20" t="s">
+      <c r="A34" s="16" t="s">
         <v>46</v>
       </c>
       <c r="B34">
         <f>covariateCoefsNew!B29</f>
-        <v>1.66</v>
+        <v>1.77</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A35" s="20" t="s">
+      <c r="A35" s="16" t="s">
         <v>47</v>
       </c>
       <c r="B35">
         <f>covariateCoefsNew!B30</f>
-        <v>1.41</v>
+        <v>1.39</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A36" s="20" t="s">
+      <c r="A36" s="16" t="s">
         <v>48</v>
       </c>
       <c r="B36">
         <f>covariateCoefsNew!B31</f>
-        <v>1.18</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A37" s="20" t="s">
+      <c r="A37" s="16" t="s">
         <v>49</v>
       </c>
       <c r="B37">
@@ -2755,43 +2755,43 @@
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A38" s="20" t="s">
+      <c r="A38" s="16" t="s">
         <v>50</v>
       </c>
       <c r="B38">
         <f>covariateCoefsNew!B33</f>
-        <v>0.89</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A39" s="20" t="s">
+      <c r="A39" s="16" t="s">
         <v>51</v>
       </c>
       <c r="B39">
         <f>covariateCoefsNew!B34</f>
-        <v>0.76</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A40" s="20" t="s">
+      <c r="A40" s="16" t="s">
         <v>52</v>
       </c>
       <c r="B40">
         <f>covariateCoefsNew!B35</f>
-        <v>1.26</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A41" s="20" t="s">
+      <c r="A41" s="16" t="s">
         <v>53</v>
       </c>
       <c r="B41">
         <f>covariateCoefsNew!B36</f>
-        <v>0.61</v>
+        <v>0.62</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A42" s="20" t="s">
+      <c r="A42" s="16" t="s">
         <v>54</v>
       </c>
       <c r="B42">
@@ -2800,89 +2800,89 @@
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A43" s="20" t="s">
+      <c r="A43" s="16" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A44" s="20" t="s">
+      <c r="A44" s="16" t="s">
         <v>56</v>
       </c>
       <c r="B44">
         <f>covariateCoefsNew!B38</f>
-        <v>0.85</v>
+        <v>1.0900000000000001</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A45" s="20" t="s">
+      <c r="A45" s="16" t="s">
         <v>57</v>
       </c>
       <c r="B45">
         <f>covariateCoefsNew!B39</f>
-        <v>0.81</v>
+        <v>1.1399999999999999</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A46" s="20" t="s">
+      <c r="A46" s="16" t="s">
         <v>58</v>
       </c>
       <c r="B46">
         <f>covariateCoefsNew!B40</f>
-        <v>0.81</v>
+        <v>1.19</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A47" s="20" t="s">
+      <c r="A47" s="16" t="s">
         <v>59</v>
       </c>
       <c r="B47">
         <f>covariateCoefsNew!B41</f>
-        <v>0.78</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A48" s="20" t="s">
+      <c r="A48" s="16" t="s">
         <v>60</v>
       </c>
       <c r="B48">
         <f>covariateCoefsNew!B42</f>
-        <v>0.82</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A49" s="20" t="s">
+      <c r="A49" s="16" t="s">
         <v>61</v>
       </c>
       <c r="B49">
         <f>covariateCoefsNew!B43</f>
-        <v>0.86</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A50" s="20" t="s">
+      <c r="A50" s="16" t="s">
         <v>62</v>
       </c>
       <c r="B50">
         <f>covariateCoefsNew!B44</f>
-        <v>0.86</v>
+        <v>1.62</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A51" s="20" t="s">
+      <c r="A51" s="16" t="s">
         <v>63</v>
       </c>
       <c r="B51">
         <f>covariateCoefsNew!B45</f>
-        <v>0.81</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="22" t="s">
+      <c r="A52" s="18" t="s">
         <v>64</v>
       </c>
       <c r="B52">
         <f>covariateCoefsNew!B46</f>
-        <v>0.86</v>
+        <v>0.84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Small updates based on submitted version - Risk of bias plot among QA studies - Slight revised bounds for ds/drtb map - clean up percentage code for cost cats and care phase - uses model from 10-13 run
</commit_message>
<xml_diff>
--- a/output/tables/covariateCoefsFormatted.xlsx
+++ b/output/tables/covariateCoefsFormatted.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hu-my.sharepoint.com/personal/nswartwood_hsph_harvard_edu/Documents/Desktop/nis100/tbPatientCosts/tb-lmic-patientcosts-review/output/tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{EDF635C7-2B95-B14A-9037-8089258CF0C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE91FC0E-F8AF-854C-9620-6566DDB68946}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{EDF635C7-2B95-B14A-9037-8089258CF0C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EBEEDFA4-6199-ED4A-BED2-0228368CC5F0}"/>
   <bookViews>
-    <workbookView xWindow="13580" yWindow="780" windowWidth="36000" windowHeight="22600" xr2:uid="{0EA54F60-3D4F-6B46-BC31-C5D89344FEF4}"/>
+    <workbookView xWindow="11820" yWindow="780" windowWidth="36000" windowHeight="22600" activeTab="1" xr2:uid="{0EA54F60-3D4F-6B46-BC31-C5D89344FEF4}"/>
   </bookViews>
   <sheets>
     <sheet name="covariateCoefsNew" sheetId="1" r:id="rId1"/>
@@ -236,7 +236,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -394,6 +394,13 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -818,7 +825,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -862,6 +869,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -930,6 +944,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1249,13 +1267,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7AB1BF8-FB56-CB4A-8B50-5BA449B6DBD0}">
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="6" max="6" width="18.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -1266,187 +1284,195 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
-        <v>0.99</v>
+        <v>1</v>
       </c>
       <c r="C2">
         <v>0.53</v>
       </c>
       <c r="D2">
-        <v>1.92</v>
+        <v>1.97</v>
       </c>
       <c r="F2" t="str">
         <f>_xlfn.CONCAT(B2, " ( ", C2, ", ", D2, ")")</f>
-        <v>0.99 ( 0.53, 1.92)</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+        <v>1 ( 0.53, 1.97)</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1.84</v>
+        <v>1.83</v>
       </c>
       <c r="C3">
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
       <c r="D3">
-        <v>3.66</v>
+        <v>3.67</v>
       </c>
       <c r="F3" t="str">
         <f t="shared" ref="F3:F46" si="0">_xlfn.CONCAT(B3, " ( ", C3, ", ", D3, ")")</f>
-        <v>1.84 ( 0.96, 3.66)</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+        <v>1.83 ( 0.95, 3.67)</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4">
-        <v>1.36</v>
+        <v>1.17</v>
       </c>
       <c r="C4">
-        <v>0.53</v>
+        <v>0.46</v>
       </c>
       <c r="D4">
-        <v>3.57</v>
+        <v>3.14</v>
       </c>
       <c r="F4" t="str">
         <f t="shared" si="0"/>
-        <v>1.36 ( 0.53, 3.57)</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+        <v>1.17 ( 0.46, 3.14)</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5">
-        <v>2.5</v>
+        <v>2.48</v>
       </c>
       <c r="C5">
-        <v>0.77</v>
+        <v>0.8</v>
       </c>
       <c r="D5">
-        <v>7.47</v>
+        <v>7.45</v>
       </c>
       <c r="F5" t="str">
         <f t="shared" si="0"/>
-        <v>2.5 ( 0.77, 7.47)</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+        <v>2.48 ( 0.8, 7.45)</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6">
-        <v>7.6</v>
-      </c>
-      <c r="C6">
-        <v>1.22</v>
-      </c>
-      <c r="D6">
-        <v>58.49</v>
-      </c>
-      <c r="F6" t="str">
-        <f t="shared" si="0"/>
-        <v>7.6 ( 1.22, 58.49)</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B6" s="19">
+        <v>7.45</v>
+      </c>
+      <c r="C6" s="19">
+        <v>1.2</v>
+      </c>
+      <c r="D6" s="19">
+        <v>62.66</v>
+      </c>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19" t="str">
+        <f t="shared" si="0"/>
+        <v>7.45 ( 1.2, 62.66)</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7">
-        <v>7.39</v>
-      </c>
-      <c r="C7">
-        <v>2.92</v>
-      </c>
-      <c r="D7">
-        <v>19.440000000000001</v>
-      </c>
-      <c r="F7" t="str">
-        <f t="shared" si="0"/>
-        <v>7.39 ( 2.92, 19.44)</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B7" s="19">
+        <v>7.42</v>
+      </c>
+      <c r="C7" s="19">
+        <v>2.9</v>
+      </c>
+      <c r="D7" s="19">
+        <v>19.399999999999999</v>
+      </c>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19" t="str">
+        <f t="shared" si="0"/>
+        <v>7.42 ( 2.9, 19.4)</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8">
-        <v>4.05</v>
-      </c>
-      <c r="C8">
-        <v>1.39</v>
-      </c>
-      <c r="D8">
-        <v>17.59</v>
-      </c>
-      <c r="F8" t="str">
-        <f t="shared" si="0"/>
-        <v>4.05 ( 1.39, 17.59)</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B8" s="19">
+        <v>4.1500000000000004</v>
+      </c>
+      <c r="C8" s="19">
+        <v>1.43</v>
+      </c>
+      <c r="D8" s="19">
+        <v>19.32</v>
+      </c>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19" t="str">
+        <f t="shared" si="0"/>
+        <v>4.15 ( 1.43, 19.32)</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9">
-        <v>6.89</v>
-      </c>
-      <c r="C9">
-        <v>2.91</v>
-      </c>
-      <c r="D9">
-        <v>17.18</v>
-      </c>
-      <c r="F9" t="str">
-        <f t="shared" si="0"/>
-        <v>6.89 ( 2.91, 17.18)</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B9" s="19">
+        <v>6.99</v>
+      </c>
+      <c r="C9" s="19">
+        <v>2.89</v>
+      </c>
+      <c r="D9" s="19">
+        <v>17.46</v>
+      </c>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19" t="str">
+        <f t="shared" si="0"/>
+        <v>6.99 ( 2.89, 17.46)</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10">
-        <v>5.92</v>
-      </c>
-      <c r="C10">
-        <v>2.5099999999999998</v>
-      </c>
-      <c r="D10">
-        <v>13.67</v>
-      </c>
-      <c r="F10" t="str">
-        <f t="shared" si="0"/>
-        <v>5.92 ( 2.51, 13.67)</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B10" s="19">
+        <v>5.86</v>
+      </c>
+      <c r="C10" s="19">
+        <v>2.41</v>
+      </c>
+      <c r="D10" s="19">
+        <v>13.69</v>
+      </c>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19" t="str">
+        <f t="shared" si="0"/>
+        <v>5.86 ( 2.41, 13.69)</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11">
-        <v>1.36</v>
+        <v>1.37</v>
       </c>
       <c r="C11">
         <v>1</v>
       </c>
       <c r="D11">
-        <v>1.89</v>
+        <v>1.9</v>
       </c>
       <c r="F11" t="str">
         <f t="shared" si="0"/>
-        <v>1.36 ( 1, 1.89)</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+        <v>1.37 ( 1, 1.9)</v>
+      </c>
+      <c r="G11">
+        <v>0.997</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1464,25 +1490,26 @@
         <v>1.1 ( 0.81, 1.48)</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13">
-        <v>1.59</v>
-      </c>
-      <c r="C13">
-        <v>1.03</v>
-      </c>
-      <c r="D13">
-        <v>2.7</v>
-      </c>
-      <c r="F13" t="str">
-        <f t="shared" si="0"/>
-        <v>1.59 ( 1.03, 2.7)</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B13" s="19">
+        <v>1.65</v>
+      </c>
+      <c r="C13" s="19">
+        <v>1.04</v>
+      </c>
+      <c r="D13" s="19">
+        <v>2.81</v>
+      </c>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19" t="str">
+        <f t="shared" si="0"/>
+        <v>1.65 ( 1.04, 2.81)</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1490,17 +1517,17 @@
         <v>1.06</v>
       </c>
       <c r="C14">
-        <v>0.61</v>
+        <v>0.59</v>
       </c>
       <c r="D14">
-        <v>1.71</v>
+        <v>1.78</v>
       </c>
       <c r="F14" t="str">
         <f t="shared" si="0"/>
-        <v>1.06 ( 0.61, 1.71)</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+        <v>1.06 ( 0.59, 1.78)</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1508,17 +1535,17 @@
         <v>1.02</v>
       </c>
       <c r="C15">
-        <v>0.4</v>
+        <v>0.38</v>
       </c>
       <c r="D15">
-        <v>1.97</v>
+        <v>2.06</v>
       </c>
       <c r="F15" t="str">
         <f t="shared" si="0"/>
-        <v>1.02 ( 0.4, 1.97)</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+        <v>1.02 ( 0.38, 2.06)</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1529,11 +1556,11 @@
         <v>0.51</v>
       </c>
       <c r="D16">
-        <v>1.55</v>
+        <v>1.56</v>
       </c>
       <c r="F16" t="str">
         <f t="shared" si="0"/>
-        <v>0.99 ( 0.51, 1.55)</v>
+        <v>0.99 ( 0.51, 1.56)</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -1541,17 +1568,17 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>1.1399999999999999</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="C17">
-        <v>0.7</v>
+        <v>0.69</v>
       </c>
       <c r="D17">
-        <v>1.85</v>
+        <v>1.9</v>
       </c>
       <c r="F17" t="str">
         <f t="shared" si="0"/>
-        <v>1.14 ( 0.7, 1.85)</v>
+        <v>1.15 ( 0.69, 1.9)</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -1559,17 +1586,17 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>1.1499999999999999</v>
+        <v>1.1599999999999999</v>
       </c>
       <c r="C18">
         <v>0.76</v>
       </c>
       <c r="D18">
-        <v>1.7</v>
+        <v>1.71</v>
       </c>
       <c r="F18" t="str">
         <f t="shared" si="0"/>
-        <v>1.15 ( 0.76, 1.7)</v>
+        <v>1.16 ( 0.76, 1.71)</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
@@ -1577,17 +1604,17 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>1.22</v>
+        <v>1.23</v>
       </c>
       <c r="C19">
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
       <c r="D19">
         <v>1.84</v>
       </c>
       <c r="F19" t="str">
         <f t="shared" si="0"/>
-        <v>1.22 ( 0.8, 1.84)</v>
+        <v>1.23 ( 0.79, 1.84)</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
@@ -1598,14 +1625,14 @@
         <v>1.36</v>
       </c>
       <c r="C20">
-        <v>0.86</v>
+        <v>0.85</v>
       </c>
       <c r="D20">
         <v>2.19</v>
       </c>
       <c r="F20" t="str">
         <f t="shared" si="0"/>
-        <v>1.36 ( 0.86, 2.19)</v>
+        <v>1.36 ( 0.85, 2.19)</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
@@ -1616,14 +1643,14 @@
         <v>1.1299999999999999</v>
       </c>
       <c r="C21">
-        <v>0.73</v>
+        <v>0.74</v>
       </c>
       <c r="D21">
-        <v>1.73</v>
+        <v>1.72</v>
       </c>
       <c r="F21" t="str">
         <f t="shared" si="0"/>
-        <v>1.13 ( 0.73, 1.73)</v>
+        <v>1.13 ( 0.74, 1.72)</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
@@ -1631,17 +1658,17 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>1.1000000000000001</v>
+        <v>1.1100000000000001</v>
       </c>
       <c r="C22">
         <v>0.68</v>
       </c>
       <c r="D22">
-        <v>1.74</v>
+        <v>1.75</v>
       </c>
       <c r="F22" t="str">
         <f t="shared" si="0"/>
-        <v>1.1 ( 0.68, 1.74)</v>
+        <v>1.11 ( 0.68, 1.75)</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
@@ -1655,11 +1682,11 @@
         <v>0.69</v>
       </c>
       <c r="D23">
-        <v>2.1</v>
+        <v>2.08</v>
       </c>
       <c r="F23" t="str">
         <f t="shared" si="0"/>
-        <v>1.18 ( 0.69, 2.1)</v>
+        <v>1.18 ( 0.69, 2.08)</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
@@ -1670,14 +1697,14 @@
         <v>1.08</v>
       </c>
       <c r="C24">
-        <v>0.54</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="D24">
-        <v>2.06</v>
+        <v>2.02</v>
       </c>
       <c r="F24" t="str">
         <f t="shared" si="0"/>
-        <v>1.08 ( 0.54, 2.06)</v>
+        <v>1.08 ( 0.55, 2.02)</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
@@ -1685,17 +1712,17 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>1.34</v>
+        <v>1.33</v>
       </c>
       <c r="C25">
         <v>0.76</v>
       </c>
       <c r="D25">
-        <v>2.72</v>
+        <v>2.71</v>
       </c>
       <c r="F25" t="str">
         <f t="shared" si="0"/>
-        <v>1.34 ( 0.76, 2.72)</v>
+        <v>1.33 ( 0.76, 2.71)</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
@@ -1706,14 +1733,14 @@
         <v>1.4</v>
       </c>
       <c r="C26">
-        <v>0.76</v>
+        <v>0.77</v>
       </c>
       <c r="D26">
-        <v>3.85</v>
+        <v>4.2300000000000004</v>
       </c>
       <c r="F26" t="str">
         <f t="shared" si="0"/>
-        <v>1.4 ( 0.76, 3.85)</v>
+        <v>1.4 ( 0.77, 4.23)</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
@@ -1724,14 +1751,14 @@
         <v>0.96</v>
       </c>
       <c r="C27">
-        <v>0.57999999999999996</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="D27">
         <v>1.54</v>
       </c>
       <c r="F27" t="str">
         <f t="shared" si="0"/>
-        <v>0.96 ( 0.58, 1.54)</v>
+        <v>0.96 ( 0.57, 1.54)</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
@@ -1742,32 +1769,33 @@
         <v>1.1399999999999999</v>
       </c>
       <c r="C28">
-        <v>0.68</v>
+        <v>0.69</v>
       </c>
       <c r="D28">
-        <v>1.86</v>
+        <v>1.88</v>
       </c>
       <c r="F28" t="str">
         <f t="shared" si="0"/>
-        <v>1.14 ( 0.68, 1.86)</v>
+        <v>1.14 ( 0.69, 1.88)</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>28</v>
       </c>
-      <c r="B29">
-        <v>1.77</v>
-      </c>
-      <c r="C29">
-        <v>1.1499999999999999</v>
-      </c>
-      <c r="D29">
+      <c r="B29" s="19">
+        <v>1.78</v>
+      </c>
+      <c r="C29" s="19">
+        <v>1.18</v>
+      </c>
+      <c r="D29" s="19">
         <v>2.72</v>
       </c>
-      <c r="F29" t="str">
-        <f t="shared" si="0"/>
-        <v>1.77 ( 1.15, 2.72)</v>
+      <c r="E29" s="19"/>
+      <c r="F29" s="19" t="str">
+        <f t="shared" si="0"/>
+        <v>1.78 ( 1.18, 2.72)</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
@@ -1781,11 +1809,11 @@
         <v>0.99</v>
       </c>
       <c r="D30">
-        <v>1.98</v>
+        <v>2</v>
       </c>
       <c r="F30" t="str">
         <f t="shared" si="0"/>
-        <v>1.39 ( 0.99, 1.98)</v>
+        <v>1.39 ( 0.99, 2)</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
@@ -1793,17 +1821,17 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>1.34</v>
+        <v>1.31</v>
       </c>
       <c r="C31">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
       <c r="D31">
-        <v>2.09</v>
+        <v>2.0299999999999998</v>
       </c>
       <c r="F31" t="str">
         <f t="shared" si="0"/>
-        <v>1.34 ( 0.85, 2.09)</v>
+        <v>1.31 ( 0.84, 2.03)</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
@@ -1814,14 +1842,14 @@
         <v>1.31</v>
       </c>
       <c r="C32">
-        <v>0.7</v>
+        <v>0.71</v>
       </c>
       <c r="D32">
-        <v>2.68</v>
+        <v>2.61</v>
       </c>
       <c r="F32" t="str">
         <f t="shared" si="0"/>
-        <v>1.31 ( 0.7, 2.68)</v>
+        <v>1.31 ( 0.71, 2.61)</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
@@ -1829,17 +1857,17 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
       <c r="C33">
-        <v>0.25</v>
+        <v>0.23</v>
       </c>
       <c r="D33">
-        <v>2.08</v>
+        <v>2.12</v>
       </c>
       <c r="F33" t="str">
         <f t="shared" si="0"/>
-        <v>0.85 ( 0.25, 2.08)</v>
+        <v>0.84 ( 0.23, 2.12)</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
@@ -1853,11 +1881,11 @@
         <v>0.45</v>
       </c>
       <c r="D34">
-        <v>1.33</v>
+        <v>1.31</v>
       </c>
       <c r="F34" t="str">
         <f t="shared" si="0"/>
-        <v>0.77 ( 0.45, 1.33)</v>
+        <v>0.77 ( 0.45, 1.31)</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
@@ -1871,11 +1899,11 @@
         <v>0.51</v>
       </c>
       <c r="D35">
-        <v>2.08</v>
+        <v>2.09</v>
       </c>
       <c r="F35" t="str">
         <f t="shared" si="0"/>
-        <v>1.03 ( 0.51, 2.08)</v>
+        <v>1.03 ( 0.51, 2.09)</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
@@ -1883,17 +1911,17 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>0.62</v>
+        <v>0.63</v>
       </c>
       <c r="C36">
         <v>0.38</v>
       </c>
       <c r="D36">
-        <v>1.18</v>
+        <v>1.17</v>
       </c>
       <c r="F36" t="str">
         <f t="shared" si="0"/>
-        <v>0.62 ( 0.38, 1.18)</v>
+        <v>0.63 ( 0.38, 1.17)</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
@@ -1907,11 +1935,11 @@
         <v>0.47</v>
       </c>
       <c r="D37">
-        <v>1.21</v>
+        <v>1.19</v>
       </c>
       <c r="F37" t="str">
         <f t="shared" si="0"/>
-        <v>0.75 ( 0.47, 1.21)</v>
+        <v>0.75 ( 0.47, 1.19)</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
@@ -1919,17 +1947,17 @@
         <v>37</v>
       </c>
       <c r="B38">
-        <v>1.0900000000000001</v>
+        <v>1.08</v>
       </c>
       <c r="C38">
         <v>0.7</v>
       </c>
       <c r="D38">
-        <v>1.7</v>
+        <v>1.69</v>
       </c>
       <c r="F38" t="str">
         <f t="shared" si="0"/>
-        <v>1.09 ( 0.7, 1.7)</v>
+        <v>1.08 ( 0.7, 1.69)</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
@@ -1943,11 +1971,11 @@
         <v>0.75</v>
       </c>
       <c r="D39">
-        <v>1.73</v>
+        <v>1.74</v>
       </c>
       <c r="F39" t="str">
         <f t="shared" si="0"/>
-        <v>1.14 ( 0.75, 1.73)</v>
+        <v>1.14 ( 0.75, 1.74)</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
@@ -1973,17 +2001,17 @@
         <v>40</v>
       </c>
       <c r="B41">
-        <v>1.17</v>
+        <v>1.1599999999999999</v>
       </c>
       <c r="C41">
         <v>0.68</v>
       </c>
       <c r="D41">
-        <v>2.1800000000000002</v>
+        <v>2.19</v>
       </c>
       <c r="F41" t="str">
         <f t="shared" si="0"/>
-        <v>1.17 ( 0.68, 2.18)</v>
+        <v>1.16 ( 0.68, 2.19)</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
@@ -1991,17 +2019,17 @@
         <v>41</v>
       </c>
       <c r="B42">
-        <v>0.81</v>
+        <v>0.82</v>
       </c>
       <c r="C42">
-        <v>0.33</v>
+        <v>0.35</v>
       </c>
       <c r="D42">
         <v>1.64</v>
       </c>
       <c r="F42" t="str">
         <f t="shared" si="0"/>
-        <v>0.81 ( 0.33, 1.64)</v>
+        <v>0.82 ( 0.35, 1.64)</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
@@ -2015,11 +2043,11 @@
         <v>0.63</v>
       </c>
       <c r="D43">
-        <v>1.65</v>
+        <v>1.67</v>
       </c>
       <c r="F43" t="str">
         <f t="shared" si="0"/>
-        <v>1.02 ( 0.63, 1.65)</v>
+        <v>1.02 ( 0.63, 1.67)</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
@@ -2027,17 +2055,17 @@
         <v>43</v>
       </c>
       <c r="B44">
-        <v>1.62</v>
+        <v>1.59</v>
       </c>
       <c r="C44">
-        <v>0.88</v>
+        <v>0.86</v>
       </c>
       <c r="D44">
-        <v>3.78</v>
+        <v>3.67</v>
       </c>
       <c r="F44" t="str">
         <f t="shared" si="0"/>
-        <v>1.62 ( 0.88, 3.78)</v>
+        <v>1.59 ( 0.86, 3.67)</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
@@ -2048,14 +2076,14 @@
         <v>0.76</v>
       </c>
       <c r="C45">
-        <v>0.46</v>
+        <v>0.45</v>
       </c>
       <c r="D45">
-        <v>1.21</v>
+        <v>1.22</v>
       </c>
       <c r="F45" t="str">
         <f t="shared" si="0"/>
-        <v>0.76 ( 0.46, 1.21)</v>
+        <v>0.76 ( 0.45, 1.22)</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
@@ -2069,11 +2097,11 @@
         <v>0.52</v>
       </c>
       <c r="D46">
-        <v>1.32</v>
+        <v>1.33</v>
       </c>
       <c r="F46" t="str">
         <f t="shared" si="0"/>
-        <v>0.84 ( 0.52, 1.32)</v>
+        <v>0.84 ( 0.52, 1.33)</v>
       </c>
     </row>
   </sheetData>
@@ -2094,17 +2122,17 @@
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="2"/>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
     </row>
     <row r="3" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="3"/>
@@ -2124,15 +2152,15 @@
       </c>
       <c r="B5" s="11" t="str">
         <f>covariateCoefsNew!F2</f>
-        <v>0.99 ( 0.53, 1.92)</v>
+        <v>1 ( 0.53, 1.97)</v>
       </c>
       <c r="C5" s="12" t="str">
         <f>covariateCoefsNew!F3</f>
-        <v>1.84 ( 0.96, 3.66)</v>
+        <v>1.83 ( 0.95, 3.67)</v>
       </c>
       <c r="D5" s="7" t="str">
         <f>covariateCoefsNew!F4</f>
-        <v>1.36 ( 0.53, 3.57)</v>
+        <v>1.17 ( 0.46, 3.14)</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -2141,15 +2169,15 @@
       </c>
       <c r="B6" s="11" t="str">
         <f>covariateCoefsNew!F11</f>
-        <v>1.36 ( 1, 1.89)</v>
+        <v>1.37 ( 1, 1.9)</v>
       </c>
       <c r="C6" s="12" t="str">
         <f>covariateCoefsNew!F12</f>
         <v>1.1 ( 0.81, 1.48)</v>
       </c>
-      <c r="D6" s="7" t="str">
+      <c r="D6" s="21" t="str">
         <f>covariateCoefsNew!F13</f>
-        <v>1.59 ( 1.03, 2.7)</v>
+        <v>1.65 ( 1.04, 2.81)</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -2158,32 +2186,32 @@
       </c>
       <c r="B7" s="11" t="str">
         <f>covariateCoefsNew!F20</f>
-        <v>1.36 ( 0.86, 2.19)</v>
+        <v>1.36 ( 0.85, 2.19)</v>
       </c>
       <c r="C7" s="12" t="str">
         <f>covariateCoefsNew!F21</f>
-        <v>1.13 ( 0.73, 1.73)</v>
+        <v>1.13 ( 0.74, 1.72)</v>
       </c>
       <c r="D7" s="7" t="str">
         <f>covariateCoefsNew!F22</f>
-        <v>1.1 ( 0.68, 1.74)</v>
+        <v>1.11 ( 0.68, 1.75)</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="11" t="str">
+      <c r="B8" s="14" t="str">
         <f>covariateCoefsNew!F29</f>
-        <v>1.77 ( 1.15, 2.72)</v>
+        <v>1.78 ( 1.18, 2.72)</v>
       </c>
       <c r="C8" s="12" t="str">
         <f>covariateCoefsNew!F30</f>
-        <v>1.39 ( 0.99, 1.98)</v>
+        <v>1.39 ( 0.99, 2)</v>
       </c>
       <c r="D8" s="7" t="str">
         <f>covariateCoefsNew!F31</f>
-        <v>1.34 ( 0.85, 2.09)</v>
+        <v>1.31 ( 0.84, 2.03)</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -2192,11 +2220,11 @@
       </c>
       <c r="B9" s="11" t="str">
         <f>covariateCoefsNew!F38</f>
-        <v>1.09 ( 0.7, 1.7)</v>
+        <v>1.08 ( 0.7, 1.69)</v>
       </c>
       <c r="C9" s="12" t="str">
         <f>covariateCoefsNew!F39</f>
-        <v>1.14 ( 0.75, 1.73)</v>
+        <v>1.14 ( 0.75, 1.74)</v>
       </c>
       <c r="D9" s="7" t="str">
         <f>covariateCoefsNew!F40</f>
@@ -2211,11 +2239,11 @@
     </row>
     <row r="11" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="20"/>
-      <c r="D11" s="22"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="25"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="3"/>
@@ -2235,15 +2263,15 @@
       </c>
       <c r="B13" s="11" t="str">
         <f>covariateCoefsNew!F5</f>
-        <v>2.5 ( 0.77, 7.47)</v>
-      </c>
-      <c r="C13" s="12" t="str">
+        <v>2.48 ( 0.8, 7.45)</v>
+      </c>
+      <c r="C13" s="20" t="str">
         <f>covariateCoefsNew!F6</f>
-        <v>7.6 ( 1.22, 58.49)</v>
-      </c>
-      <c r="D13" s="7" t="str">
+        <v>7.45 ( 1.2, 62.66)</v>
+      </c>
+      <c r="D13" s="21" t="str">
         <f>covariateCoefsNew!F7</f>
-        <v>7.39 ( 2.92, 19.44)</v>
+        <v>7.42 ( 2.9, 19.4)</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
@@ -2252,15 +2280,15 @@
       </c>
       <c r="B14" s="11" t="str">
         <f>covariateCoefsNew!F14</f>
-        <v>1.06 ( 0.61, 1.71)</v>
+        <v>1.06 ( 0.59, 1.78)</v>
       </c>
       <c r="C14" s="12" t="str">
         <f>covariateCoefsNew!F15</f>
-        <v>1.02 ( 0.4, 1.97)</v>
+        <v>1.02 ( 0.38, 2.06)</v>
       </c>
       <c r="D14" s="7" t="str">
         <f>covariateCoefsNew!F16</f>
-        <v>0.99 ( 0.51, 1.55)</v>
+        <v>0.99 ( 0.51, 1.56)</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
@@ -2269,15 +2297,15 @@
       </c>
       <c r="B15" s="11" t="str">
         <f>covariateCoefsNew!F23</f>
-        <v>1.18 ( 0.69, 2.1)</v>
+        <v>1.18 ( 0.69, 2.08)</v>
       </c>
       <c r="C15" s="12" t="str">
         <f>covariateCoefsNew!F24</f>
-        <v>1.08 ( 0.54, 2.06)</v>
+        <v>1.08 ( 0.55, 2.02)</v>
       </c>
       <c r="D15" s="7" t="str">
         <f>covariateCoefsNew!F25</f>
-        <v>1.34 ( 0.76, 2.72)</v>
+        <v>1.33 ( 0.76, 2.71)</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
@@ -2286,15 +2314,15 @@
       </c>
       <c r="B16" s="11" t="str">
         <f>covariateCoefsNew!F32</f>
-        <v>1.31 ( 0.7, 2.68)</v>
+        <v>1.31 ( 0.71, 2.61)</v>
       </c>
       <c r="C16" s="12" t="str">
         <f>covariateCoefsNew!F33</f>
-        <v>0.85 ( 0.25, 2.08)</v>
+        <v>0.84 ( 0.23, 2.12)</v>
       </c>
       <c r="D16" s="7" t="str">
         <f>covariateCoefsNew!F34</f>
-        <v>0.77 ( 0.45, 1.33)</v>
+        <v>0.77 ( 0.45, 1.31)</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
@@ -2303,15 +2331,15 @@
       </c>
       <c r="B17" s="11" t="str">
         <f>covariateCoefsNew!F41</f>
-        <v>1.17 ( 0.68, 2.18)</v>
+        <v>1.16 ( 0.68, 2.19)</v>
       </c>
       <c r="C17" s="12" t="str">
         <f>covariateCoefsNew!F42</f>
-        <v>0.81 ( 0.33, 1.64)</v>
+        <v>0.82 ( 0.35, 1.64)</v>
       </c>
       <c r="D17" s="7" t="str">
         <f>covariateCoefsNew!F43</f>
-        <v>1.02 ( 0.63, 1.65)</v>
+        <v>1.02 ( 0.63, 1.67)</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -2322,11 +2350,11 @@
     </row>
     <row r="19" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
-      <c r="B19" s="21" t="s">
+      <c r="B19" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="C19" s="20"/>
-      <c r="D19" s="22"/>
+      <c r="C19" s="23"/>
+      <c r="D19" s="25"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="3"/>
@@ -2344,17 +2372,17 @@
       <c r="A21" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B21" s="11" t="str">
+      <c r="B21" s="14" t="str">
         <f>covariateCoefsNew!F8</f>
-        <v>4.05 ( 1.39, 17.59)</v>
-      </c>
-      <c r="C21" s="12" t="str">
+        <v>4.15 ( 1.43, 19.32)</v>
+      </c>
+      <c r="C21" s="20" t="str">
         <f>covariateCoefsNew!F9</f>
-        <v>6.89 ( 2.91, 17.18)</v>
-      </c>
-      <c r="D21" s="7" t="str">
+        <v>6.99 ( 2.89, 17.46)</v>
+      </c>
+      <c r="D21" s="21" t="str">
         <f>covariateCoefsNew!F10</f>
-        <v>5.92 ( 2.51, 13.67)</v>
+        <v>5.86 ( 2.41, 13.69)</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
@@ -2363,15 +2391,15 @@
       </c>
       <c r="B22" s="11" t="str">
         <f>covariateCoefsNew!F17</f>
-        <v>1.14 ( 0.7, 1.85)</v>
+        <v>1.15 ( 0.69, 1.9)</v>
       </c>
       <c r="C22" s="12" t="str">
         <f>covariateCoefsNew!F18</f>
-        <v>1.15 ( 0.76, 1.7)</v>
+        <v>1.16 ( 0.76, 1.71)</v>
       </c>
       <c r="D22" s="7" t="str">
         <f>covariateCoefsNew!F19</f>
-        <v>1.22 ( 0.8, 1.84)</v>
+        <v>1.23 ( 0.79, 1.84)</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
@@ -2380,15 +2408,15 @@
       </c>
       <c r="B23" s="11" t="str">
         <f>covariateCoefsNew!F26</f>
-        <v>1.4 ( 0.76, 3.85)</v>
+        <v>1.4 ( 0.77, 4.23)</v>
       </c>
       <c r="C23" s="12" t="str">
         <f>covariateCoefsNew!F27</f>
-        <v>0.96 ( 0.58, 1.54)</v>
+        <v>0.96 ( 0.57, 1.54)</v>
       </c>
       <c r="D23" s="7" t="str">
         <f>covariateCoefsNew!F28</f>
-        <v>1.14 ( 0.68, 1.86)</v>
+        <v>1.14 ( 0.69, 1.88)</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
@@ -2397,15 +2425,15 @@
       </c>
       <c r="B24" s="11" t="str">
         <f>covariateCoefsNew!F35</f>
-        <v>1.03 ( 0.51, 2.08)</v>
+        <v>1.03 ( 0.51, 2.09)</v>
       </c>
       <c r="C24" s="12" t="str">
         <f>covariateCoefsNew!F36</f>
-        <v>0.62 ( 0.38, 1.18)</v>
+        <v>0.63 ( 0.38, 1.17)</v>
       </c>
       <c r="D24" s="7" t="str">
         <f>covariateCoefsNew!F37</f>
-        <v>0.75 ( 0.47, 1.21)</v>
+        <v>0.75 ( 0.47, 1.19)</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -2414,15 +2442,15 @@
       </c>
       <c r="B25" s="15" t="str">
         <f>covariateCoefsNew!F44</f>
-        <v>1.62 ( 0.88, 3.78)</v>
+        <v>1.59 ( 0.86, 3.67)</v>
       </c>
       <c r="C25" s="8" t="str">
         <f>covariateCoefsNew!F45</f>
-        <v>0.76 ( 0.46, 1.21)</v>
+        <v>0.76 ( 0.45, 1.22)</v>
       </c>
       <c r="D25" s="9" t="str">
         <f>covariateCoefsNew!F46</f>
-        <v>0.84 ( 0.52, 1.32)</v>
+        <v>0.84 ( 0.52, 1.33)</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
@@ -2461,7 +2489,7 @@
       </c>
       <c r="B3">
         <f>covariateCoefsNew!B2</f>
-        <v>0.99</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -2470,7 +2498,7 @@
       </c>
       <c r="B4">
         <f>covariateCoefsNew!B3</f>
-        <v>1.84</v>
+        <v>1.83</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -2479,7 +2507,7 @@
       </c>
       <c r="B5">
         <f>covariateCoefsNew!B4</f>
-        <v>1.36</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -2488,7 +2516,7 @@
       </c>
       <c r="B6">
         <f>covariateCoefsNew!B5</f>
-        <v>2.5</v>
+        <v>2.48</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -2497,7 +2525,7 @@
       </c>
       <c r="B7">
         <f>covariateCoefsNew!B6</f>
-        <v>7.6</v>
+        <v>7.45</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -2506,7 +2534,7 @@
       </c>
       <c r="B8">
         <f>covariateCoefsNew!B7</f>
-        <v>7.39</v>
+        <v>7.42</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -2515,7 +2543,7 @@
       </c>
       <c r="B9">
         <f>covariateCoefsNew!B8</f>
-        <v>4.05</v>
+        <v>4.1500000000000004</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -2524,7 +2552,7 @@
       </c>
       <c r="B10">
         <f>covariateCoefsNew!B9</f>
-        <v>6.89</v>
+        <v>6.99</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -2533,7 +2561,7 @@
       </c>
       <c r="B11">
         <f>covariateCoefsNew!B10</f>
-        <v>5.92</v>
+        <v>5.86</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
@@ -2547,7 +2575,7 @@
       </c>
       <c r="B13">
         <f>covariateCoefsNew!B11</f>
-        <v>1.36</v>
+        <v>1.37</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
@@ -2565,7 +2593,7 @@
       </c>
       <c r="B15">
         <f>covariateCoefsNew!B13</f>
-        <v>1.59</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
@@ -2601,7 +2629,7 @@
       </c>
       <c r="B19">
         <f>covariateCoefsNew!B17</f>
-        <v>1.1399999999999999</v>
+        <v>1.1499999999999999</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
@@ -2610,7 +2638,7 @@
       </c>
       <c r="B20">
         <f>covariateCoefsNew!B18</f>
-        <v>1.1499999999999999</v>
+        <v>1.1599999999999999</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
@@ -2619,7 +2647,7 @@
       </c>
       <c r="B21">
         <f>covariateCoefsNew!B19</f>
-        <v>1.22</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
@@ -2656,7 +2684,7 @@
       </c>
       <c r="B26">
         <f>covariateCoefsNew!B22</f>
-        <v>1.1000000000000001</v>
+        <v>1.1100000000000001</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
@@ -2683,7 +2711,7 @@
       </c>
       <c r="B29">
         <f>covariateCoefsNew!B25</f>
-        <v>1.34</v>
+        <v>1.33</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
@@ -2724,7 +2752,7 @@
       </c>
       <c r="B34">
         <f>covariateCoefsNew!B29</f>
-        <v>1.77</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
@@ -2742,7 +2770,7 @@
       </c>
       <c r="B36">
         <f>covariateCoefsNew!B31</f>
-        <v>1.34</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
@@ -2760,7 +2788,7 @@
       </c>
       <c r="B38">
         <f>covariateCoefsNew!B33</f>
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
@@ -2787,7 +2815,7 @@
       </c>
       <c r="B41">
         <f>covariateCoefsNew!B36</f>
-        <v>0.62</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
@@ -2810,7 +2838,7 @@
       </c>
       <c r="B44">
         <f>covariateCoefsNew!B38</f>
-        <v>1.0900000000000001</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
@@ -2837,7 +2865,7 @@
       </c>
       <c r="B47">
         <f>covariateCoefsNew!B41</f>
-        <v>1.17</v>
+        <v>1.1599999999999999</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
@@ -2846,7 +2874,7 @@
       </c>
       <c r="B48">
         <f>covariateCoefsNew!B42</f>
-        <v>0.81</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
@@ -2864,7 +2892,7 @@
       </c>
       <c r="B50">
         <f>covariateCoefsNew!B44</f>
-        <v>1.62</v>
+        <v>1.59</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>